<commit_message>
CASE_PUMPBTC: DRIP-WATCH trigger + NOISE-DRIP-WATCH event (20/08)
TRIGGERS row 2 (ACTIVE):
  DRIP-WATCH 2026-08-20
  Observation: List B drip pos +17%/13d · div_avg3 +0.064 từ đáy
    (0.184@Jul23 → 0.248@Aug06) · struct_n=51 · dưới threshold registry 10×
  Escalate condition (bất kỳ 1 của 4):
    (1) div_avg3 ≥ 0.35
    (2) pos_r +15%/2d
    (3) gLSR flush ≥30%/3d
    (4) episode break (div > 0.5 liên tiếp ≥3d = E-R1(a))
  Action: alert operator đọc lại + candidate vào unhedge_registry nếu (4)

EVENTS row 11 (unresolved):
  2026-08-17→2026-08-20 · NOISE-DRIP-WATCH
  List B report chuỗi 4d: drip dưới ngưỡng registry E-R1 10×
  (drift cần ≥+0.15/7d, current +0.064/13d = ~5× dưới)
  Classified NOISE — không đủ signal vào unhedge_registry, đủ signal
  đặt DRIP-WATCH trigger chờ escalation
  Ref: operator relay 20/08 + watchlist_log v1.4 List B

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_PUMPBTC.xlsx
+++ b/docs/case_files/CASE_PUMPBTC.xlsx
@@ -551,7 +551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I75"/>
+  <dimension ref="A1:B72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="22" customWidth="1" style="10" min="1" max="1"/>
@@ -804,7 +804,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
@@ -860,7 +859,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
@@ -916,7 +914,6 @@
         </is>
       </c>
     </row>
-    <row r="36"/>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
@@ -972,7 +969,6 @@
         </is>
       </c>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
@@ -1040,7 +1036,6 @@
         </is>
       </c>
     </row>
-    <row r="49"/>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
@@ -1108,7 +1103,6 @@
         </is>
       </c>
     </row>
-    <row r="56"/>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
@@ -1140,7 +1134,6 @@
         </is>
       </c>
     </row>
-    <row r="60"/>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
@@ -1208,7 +1201,6 @@
         </is>
       </c>
     </row>
-    <row r="67"/>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
@@ -1264,9 +1256,6 @@
         </is>
       </c>
     </row>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8206,7 +8195,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" customWidth="1" style="10" min="1" max="2"/>
@@ -8485,11 +8474,31 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="n"/>
-      <c r="B11" s="8" t="n"/>
-      <c r="C11" s="8" t="n"/>
-      <c r="D11" s="8" t="n"/>
-      <c r="E11" s="8" t="n"/>
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>2026-08-17→2026-08-20</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>NOISE-DRIP-WATCH</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>List B report chuỗi 17-20/08 (4d liên tiếp): drip pos +17%/13d + div_avg3 +0.064 từ đáy episode. Dưới ngưỡng registry E-R1 10× (drift threshold cần ≥+0.15/7d, current +0.064/13d = ~5× dưới ngưỡng). Classified NOISE-DRIP-WATCH — không đủ signal vào unhedge_registry, nhưng đủ signal đặt trigger DRIP-WATCH (§TRIGGERS row 2) chờ escalation.</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>operator relay 20/08 + watchlist_log v1.4 List B</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>unresolved</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="n"/>
@@ -8712,13 +8721,70 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>TRIGGERS (PUMPBTC) — PENDING operator to define</t>
+          <t>trigger_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>date_opened</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>observation</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>escalate_condition</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>action_if_triggered</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>DRIP-WATCH</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>List B drip pos +17%/13d · div_avg3 +0.064 từ đáy episode (0.184@Jul23 → 0.248@Aug06 range) · struct_n=51 · vẫn dưới threshold registry 10× (fw-139 backfill 0 rows PUMPBTC)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Nâng cấp thành alert đọc lại khi bất kỳ: (1) div_avg3 ≥ 0.35  · (2) pos_r +15%/2d  · (3) gLSR flush ≥30%/3d  · (4) episode break (div &gt; 0.5 liên tiếp ≥3d = E-R1(a))</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Alert operator đọc lại + candidate vào unhedge_registry E-R7 nếu (4) fires</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
     </row>
@@ -8733,7 +8799,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -8754,7 +8820,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -8775,7 +8841,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">

</xml_diff>